<commit_message>
Add individual CSV datasets for each problem and set Problem 1 as first sheet in Excel
</commit_message>
<xml_diff>
--- a/Jamovi_Seatwork_Practice_Data.xlsx
+++ b/Jamovi_Seatwork_Practice_Data.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory &amp; Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_1_Seatwork1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_2_Seatwork2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_3_OneWay_ANOVA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_4_TwoWay_ANOVA" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_5_Variance_Descriptives" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_1_Seatwork1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_2_Seatwork2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_3_OneWay_ANOVA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_4_TwoWay_ANOVA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problem_5_Variance_Descriptives" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory &amp; Guide" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook_and_Scales" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -522,354 +522,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PROBABILITY &amp; STATISTICS - FRESH PRACTICE PROBLEM SET DATASETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>New, fresh datasets calibrated for Seatwork Problems 1 through 5. Each tab contains clean numerical codes and text ranges for immediate Jamovi analysis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tab Name</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Problem Title &amp; Coverage</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Statistical Test in Jamovi</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Jamovi Menu Navigation</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Independent Variable (IV)</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Dependent Variable (DV)</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Expected Statistical Outputs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="75" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Problem_1_Seatwork1</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Problem 1 (Seatwork 1 Format): Digital Learning Engagement &amp; Academic Stress</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>• Frequencies &amp; Percentages
-• Kruskal-Wallis (Age, Year Level, Allowance)
-• Mann-Whitney U (Gender)
-• Spearman's Rho Correlation</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>1. Analyses -&gt; Exploration -&gt; Descriptives (Demographics)
-2. Analyses -&gt; ANOVA -&gt; One-Way ANOVA (check Kruskal-Wallis)
-3. Analyses -&gt; T-Tests -&gt; Independent Samples (check Mann-Whitney U)
-4. Analyses -&gt; Regression -&gt; Correlation Matrix (check Spearman)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Demographics: Age_Bracket, Gender, Year_Level, Monthly_Allowance
-Digital Learning Engagement (Continuous)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Academic Stress (Continuous Likert Composite)</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>• Demographic tables (f and %)
-• Kruskal-Wallis: Age χ²=0.908 (p=.823), Year Level χ²=0.458 (p=.928), Allowance χ²=0.312 (p=.855)
-• Mann-Whitney U=2762.0 (p=.724)
-• Spearman's rho=0.294*** (p&lt;.001)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="75" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Problem_2_Seatwork2</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Problem 2 (Seatwork 2 Format): Digital Resource Utilization, Collaborative Peer Learning &amp; Statistical Competency</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>• Pearson Correlation Matrix (3 bivariate relationships)
-• Simple Linear Regression (Peer Learning predicting Competency)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>1. Analyses -&gt; Regression -&gt; Correlation Matrix (drag DRU, CPL, SC; check Pearson &amp; Report Significance)
-2. Analyses -&gt; Regression -&gt; Linear Regression (Dependent: Statistical_Competency; Covariate: Peer_Learning; check R, R², Model Coefficients)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>IV1: Digital Resource Utilization (DRU)
-IV2: Collaborative Peer Learning (CPL)</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>DV1: Collaborative Peer Learning
-DV2: Statistical Competency (SC)</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>• r(DRU, SC) = 0.380 (Low positive, p&lt;.001, Reject H0)
-• r(DRU, CPL) = 0.571 (Moderate positive, p&lt;.001, Reject H0)
-• r(CPL, SC) = 0.444 (Moderate positive, p&lt;.001, Reject H0)
-• Regression: Intercept=2.117, Slope=0.399, R=0.444, R²=0.197, F=45.1, p&lt;.001 (Reject H0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="75" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Problem_3_OneWay_ANOVA</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Problem 3 (Reviewer Format): Statistical Competency Across 4 Academic Programs</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>• One-Way ANOVA (Fisher's &amp; Welch's)
-• Descriptives (Means &amp; SDs)
-• Post-Hoc Test (Tukey HSD)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Analyses -&gt; ANOVA -&gt; One-Way ANOVA
-• Dependent Variable: Statistical_Competency_Score
-• Grouping Variable: Academic_Program
-• Variances: Don't assume equal (Welch's) / Assume equal (Fisher's)
-• Check Descriptives table &amp; Tukey Post-Hoc</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Academic_Program (Computing &amp; IT, Engineering, Business &amp; Accountancy, Arts &amp; Sciences)</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Statistical_Competency_Score (Continuous 0-100 scale)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>• Overall ANOVA: F(3, 116) = 68.59, p &lt; .001 (Significant -&gt; Reject H0)
-• Group Means: Engineering (83.5), Computing (76.0), Business (68.5), Arts (61.0)
-• Tukey Post-Hoc: All pairwise differences significant (p &lt; .05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Problem_4_TwoWay_ANOVA</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Problem 4 (Reviewer Format): Instructional Mode &amp; Math Background on Exam Performance</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>• Two-Way ANOVA (Factorial ANOVA)
-• Main Effects &amp; Interaction Effect
-• Post-Hoc Tests &amp; Estimated Marginal Means Plot</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Analyses -&gt; ANOVA -&gt; ANOVA
-• Dependent Variable: Exam_Score
-• Fixed Factors: Instructional_Mode, Math_Background
-• Post Hoc Tests: Drag factors to right box
-• Estimated Marginal Means: Drag factors to display box</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Factor A: Instructional_Mode (Traditional Lecture, Blended Learning, Gamified Active Learning)
-Factor B: Math_Background (Non-STEM, STEM)</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Exam_Score (Continuous 0-100 scale)</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>• Main Effect (Instructional_Mode): Significant (p &lt; .001)
-• Main Effect (Math_Background): Significant (p &lt; .001)
-• Interaction Effect (Mode * Background): Significant (p &lt; .05)
-• Interaction Plot: Displays non-parallel interaction lines</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Problem_5_Variance_Descriptives</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Problem 5 (Reviewer Format): Performance Consistency Between Two Learning Cohorts</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>• Exploration -&gt; Descriptives
-• Central Tendency: Mean, Median
-• Dispersion: Variance, Std. Deviation, IQR, Range</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Analyses -&gt; Exploration -&gt; Descriptives
-• Variables: Quiz_Score, Weekly_Study_Hours
-• Split by: Section (Section Alpha vs Section Beta)
-• Under Central Tendency: check Mean, Median
-• Under Dispersion: check Variance, Std. deviation, IQR, Min, Max</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Section (Section Alpha [Traditional Study] vs Section Beta [Peer Study])</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Quiz_Score (Continuous), Weekly_Study_Hours (Continuous)</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>• Section Alpha: Mean=77.2, Variance=163.3, SD=12.8 (High dispersion / Inconsistent)
-• Section Beta: Mean=78.4, Variance=26.0, SD=5.1 (Low dispersion / Highly Consistent)
-• Section Beta demonstrates far superior consistency!</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="75" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Codebook_and_Scales</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Questionnaire Coding Scheme, Variable Types &amp; Interpretation Benchmarks</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Jamovi Setup Reference: Variable Measure Types and Numerical Code to Text Label Mapping</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Double-click column header in Jamovi to verify:
-• Measure Type: Continuous 123, Nominal, or Ordinal
-• Values &amp; Labels: e.g. 1 = Male, 2 = Female</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>All Survey Variables</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>All Survey Variables</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>• Complete variable dictionary with text ranges
-• Ms. Lugo's Correlation Interpretation Table (±1.00 to 0.00)
-• p-value Significance &amp; Null Hypothesis Decision Table
-• 4-Point &amp; 5-Point Likert Scale Verbal Interpretation Scales</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8154,7 +7806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14736,7 +14388,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18036,7 +17688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20970,7 +20622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22940,6 +22592,354 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROBABILITY &amp; STATISTICS - FRESH PRACTICE PROBLEM SET DATASETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>New, fresh datasets calibrated for Seatwork Problems 1 through 5. Each tab contains clean numerical codes and text ranges for immediate Jamovi analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tab Name</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Problem Title &amp; Coverage</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Statistical Test in Jamovi</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Jamovi Menu Navigation</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Independent Variable (IV)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Dependent Variable (DV)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Expected Statistical Outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Problem_1_Seatwork1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Problem 1 (Seatwork 1 Format): Digital Learning Engagement &amp; Academic Stress</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>• Frequencies &amp; Percentages
+• Kruskal-Wallis (Age, Year Level, Allowance)
+• Mann-Whitney U (Gender)
+• Spearman's Rho Correlation</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1. Analyses -&gt; Exploration -&gt; Descriptives (Demographics)
+2. Analyses -&gt; ANOVA -&gt; One-Way ANOVA (check Kruskal-Wallis)
+3. Analyses -&gt; T-Tests -&gt; Independent Samples (check Mann-Whitney U)
+4. Analyses -&gt; Regression -&gt; Correlation Matrix (check Spearman)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Demographics: Age_Bracket, Gender, Year_Level, Monthly_Allowance
+Digital Learning Engagement (Continuous)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Academic Stress (Continuous Likert Composite)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>• Demographic tables (f and %)
+• Kruskal-Wallis: Age χ²=0.908 (p=.823), Year Level χ²=0.458 (p=.928), Allowance χ²=0.312 (p=.855)
+• Mann-Whitney U=2762.0 (p=.724)
+• Spearman's rho=0.294*** (p&lt;.001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Problem_2_Seatwork2</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Problem 2 (Seatwork 2 Format): Digital Resource Utilization, Collaborative Peer Learning &amp; Statistical Competency</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>• Pearson Correlation Matrix (3 bivariate relationships)
+• Simple Linear Regression (Peer Learning predicting Competency)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>1. Analyses -&gt; Regression -&gt; Correlation Matrix (drag DRU, CPL, SC; check Pearson &amp; Report Significance)
+2. Analyses -&gt; Regression -&gt; Linear Regression (Dependent: Statistical_Competency; Covariate: Peer_Learning; check R, R², Model Coefficients)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>IV1: Digital Resource Utilization (DRU)
+IV2: Collaborative Peer Learning (CPL)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>DV1: Collaborative Peer Learning
+DV2: Statistical Competency (SC)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>• r(DRU, SC) = 0.380 (Low positive, p&lt;.001, Reject H0)
+• r(DRU, CPL) = 0.571 (Moderate positive, p&lt;.001, Reject H0)
+• r(CPL, SC) = 0.444 (Moderate positive, p&lt;.001, Reject H0)
+• Regression: Intercept=2.117, Slope=0.399, R=0.444, R²=0.197, F=45.1, p&lt;.001 (Reject H0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Problem_3_OneWay_ANOVA</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Problem 3 (Reviewer Format): Statistical Competency Across 4 Academic Programs</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>• One-Way ANOVA (Fisher's &amp; Welch's)
+• Descriptives (Means &amp; SDs)
+• Post-Hoc Test (Tukey HSD)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Analyses -&gt; ANOVA -&gt; One-Way ANOVA
+• Dependent Variable: Statistical_Competency_Score
+• Grouping Variable: Academic_Program
+• Variances: Don't assume equal (Welch's) / Assume equal (Fisher's)
+• Check Descriptives table &amp; Tukey Post-Hoc</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Academic_Program (Computing &amp; IT, Engineering, Business &amp; Accountancy, Arts &amp; Sciences)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Statistical_Competency_Score (Continuous 0-100 scale)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>• Overall ANOVA: F(3, 116) = 68.59, p &lt; .001 (Significant -&gt; Reject H0)
+• Group Means: Engineering (83.5), Computing (76.0), Business (68.5), Arts (61.0)
+• Tukey Post-Hoc: All pairwise differences significant (p &lt; .05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Problem_4_TwoWay_ANOVA</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Problem 4 (Reviewer Format): Instructional Mode &amp; Math Background on Exam Performance</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>• Two-Way ANOVA (Factorial ANOVA)
+• Main Effects &amp; Interaction Effect
+• Post-Hoc Tests &amp; Estimated Marginal Means Plot</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Analyses -&gt; ANOVA -&gt; ANOVA
+• Dependent Variable: Exam_Score
+• Fixed Factors: Instructional_Mode, Math_Background
+• Post Hoc Tests: Drag factors to right box
+• Estimated Marginal Means: Drag factors to display box</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Factor A: Instructional_Mode (Traditional Lecture, Blended Learning, Gamified Active Learning)
+Factor B: Math_Background (Non-STEM, STEM)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Exam_Score (Continuous 0-100 scale)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>• Main Effect (Instructional_Mode): Significant (p &lt; .001)
+• Main Effect (Math_Background): Significant (p &lt; .001)
+• Interaction Effect (Mode * Background): Significant (p &lt; .05)
+• Interaction Plot: Displays non-parallel interaction lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Problem_5_Variance_Descriptives</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Problem 5 (Reviewer Format): Performance Consistency Between Two Learning Cohorts</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>• Exploration -&gt; Descriptives
+• Central Tendency: Mean, Median
+• Dispersion: Variance, Std. Deviation, IQR, Range</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Analyses -&gt; Exploration -&gt; Descriptives
+• Variables: Quiz_Score, Weekly_Study_Hours
+• Split by: Section (Section Alpha vs Section Beta)
+• Under Central Tendency: check Mean, Median
+• Under Dispersion: check Variance, Std. deviation, IQR, Min, Max</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Section (Section Alpha [Traditional Study] vs Section Beta [Peer Study])</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Quiz_Score (Continuous), Weekly_Study_Hours (Continuous)</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>• Section Alpha: Mean=77.2, Variance=163.3, SD=12.8 (High dispersion / Inconsistent)
+• Section Beta: Mean=78.4, Variance=26.0, SD=5.1 (Low dispersion / Highly Consistent)
+• Section Beta demonstrates far superior consistency!</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Codebook_and_Scales</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Questionnaire Coding Scheme, Variable Types &amp; Interpretation Benchmarks</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Jamovi Setup Reference: Variable Measure Types and Numerical Code to Text Label Mapping</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Double-click column header in Jamovi to verify:
+• Measure Type: Continuous 123, Nominal, or Ordinal
+• Values &amp; Labels: e.g. 1 = Male, 2 = Female</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>All Survey Variables</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>All Survey Variables</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>• Complete variable dictionary with text ranges
+• Ms. Lugo's Correlation Interpretation Table (±1.00 to 0.00)
+• p-value Significance &amp; Null Hypothesis Decision Table
+• 4-Point &amp; 5-Point Likert Scale Verbal Interpretation Scales</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22967,7 +22967,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -23239,8 +23238,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>

</xml_diff>